<commit_message>
Fix J05/J07 buildings, label highlighted footprints, reposition controls
- Correct J05 (Workshop building) and J07 (Mechanical Engineering/AMME)
  coordinates — previously J05 duplicated J03's location, so their pins shared
  a building. Validated other footprints (all within ~30m of their points).
- Centre pins/hubs on the real footprint centroid so they sit on the building.
- Add a building-code label (e.g. "J03") in dark ochre under each highlighted
  building, via a symbol layer on the footprints (codes from the Buildings sheet).
- Float the top-right map controls left of the index panel so they no longer
  overlap (controls return to the edge on mobile, where the index is a bottom sheet).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSS-CRF-MapData.xlsx
+++ b/TSS-CRF-MapData.xlsx
@@ -1034,10 +1034,10 @@
         </is>
       </c>
       <c r="D10" s="26" t="n">
-        <v>-33.8893</v>
+        <v>-33.889268</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>151.1925</v>
+        <v>151.194174</v>
       </c>
       <c r="F10" s="25" t="inlineStr">
         <is>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="G10" s="25" t="inlineStr">
         <is>
-          <t>Estimate — verify</t>
+          <t>OSM 'Mechanical Engineering' building (AMME) — verify</t>
         </is>
       </c>
     </row>
@@ -1067,10 +1067,10 @@
         </is>
       </c>
       <c r="D11" s="26" t="n">
-        <v>-33.890141</v>
+        <v>-33.891151</v>
       </c>
       <c r="E11" s="26" t="n">
-        <v>151.193116</v>
+        <v>151.193632</v>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="G11" s="25" t="inlineStr">
         <is>
-          <t>Estimate (near PNR) — verify</t>
+          <t>OSM 'Workshop' building, Darlington — verify</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,6 @@
           <t>Centenary Institute</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" s="24" t="n">
         <v>-33.888086</v>
       </c>
@@ -1185,7 +1184,6 @@
           <t>Kolling Institute</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" s="24" t="n">
         <v>-33.820579</v>
       </c>
@@ -1214,7 +1212,6 @@
           <t>Royal North Shore Hospital</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" s="24" t="n">
         <v>-33.821432</v>
       </c>
@@ -1272,7 +1269,6 @@
           <t>Biomedical Building, ATP</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" s="24" t="n">
         <v>-33.896263</v>
       </c>
@@ -1301,7 +1297,6 @@
           <t>Moore Theological College</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" s="24" t="n">
         <v>-33.891704</v>
       </c>
@@ -1359,7 +1354,6 @@
           <t>Geoscience</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
       <c r="D21" s="24" t="n"/>
       <c r="E21" s="24" t="n"/>
       <c r="F21" t="inlineStr">

</xml_diff>

<commit_message>
Area-weighted centroids, fixed building labels, fan-out default, dedupe
- Fix footprint centroid to area-weighted (was vertex-average), so hubs/pins sit
  at the true building centre.
- Building-code labels are now fixed-coordinate points (no zoom-dependent offset):
  centred on multi-facility buildings (pins fan around the centre), just below the
  pin on single-facility ones. New facility-labels source/layer.
- Make fan-out the default overlap mode while spider UX is refined.
- Duplicate-building fixes: relocate Sydney Institute of Agriculture (was on A31's
  footprint) to R. D. Watt Building. No two coded buildings now share a location.
- Expand CLAUDE.md: full status, file layout/modules, conventions, caveats.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TSS-CRF-MapData.xlsx
+++ b/TSS-CRF-MapData.xlsx
@@ -1242,10 +1242,10 @@
       </c>
       <c r="C17" s="25" t="inlineStr"/>
       <c r="D17" s="26" t="n">
-        <v>-33.8885</v>
+        <v>-33.885467</v>
       </c>
       <c r="E17" s="26" t="n">
-        <v>151.1875</v>
+        <v>151.185549</v>
       </c>
       <c r="F17" s="25" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="G17" s="25" t="inlineStr">
         <is>
-          <t>Placeholder at campus — verify</t>
+          <t>R. D. Watt Building (Institute of Agriculture base) — distributed, verify</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix building footprint matching: support multipolygon relations, fix centroid precision for small footprints
Madsen (F09) and other small/relation-mapped buildings were rendering with
wrong/offset footprints because build-footprints.mjs only queried
way["building"] (missing relation["building"] multipolygons) and its
centroid calc lost precision on tiny polygons due to coordinate cancellation.
</commit_message>
<xml_diff>
--- a/TSS-CRF-MapData.xlsx
+++ b/TSS-CRF-MapData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rbar3075/Claude/Usyd/UsydMapTSS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{708FD983-AF10-FC42-B2CC-E8603CBC4201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DCFC3D4-DBBD-2840-8395-10CBFA1D2A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34980" yWindow="-31380" windowWidth="51200" windowHeight="31400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-34980" yWindow="-31400" windowWidth="51200" windowHeight="31400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="831" uniqueCount="209">
   <si>
     <t>Map Label</t>
   </si>
@@ -646,6 +646,27 @@
   </si>
   <si>
     <t>https://www.sydney.edu.au/science/about/locations-and-facilities/research-facilities/chemistry-facilities.html</t>
+  </si>
+  <si>
+    <t>sydney.edu.au/research/facilities/sydney-microscopy-and-microanalysis.html</t>
+  </si>
+  <si>
+    <t>sydney.edu.au/research/facilities/sydney-imaging.html</t>
+  </si>
+  <si>
+    <t>sydney.edu.au/research/facilities/sydney-analytical.html</t>
+  </si>
+  <si>
+    <t>sydney.edu.au/research/facilities/sydney-mass-spectrometry.html</t>
+  </si>
+  <si>
+    <t>sydney.edu.au/research/facilities/sydney-informatics-hub.html</t>
+  </si>
+  <si>
+    <t>sydney.edu.au/research/facilities/sydney-manufacturing-hub.html</t>
+  </si>
+  <si>
+    <t>sydney.edu.au/research/facilities/sydney-nano-foundry.html</t>
   </si>
 </sst>
 </file>
@@ -1956,7 +1977,7 @@
         <v>41</v>
       </c>
       <c r="O5" t="s">
-        <v>42</v>
+        <v>202</v>
       </c>
     </row>
     <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2000,7 +2021,7 @@
         <v>24</v>
       </c>
       <c r="O6" t="s">
-        <v>42</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2044,7 +2065,7 @@
         <v>24</v>
       </c>
       <c r="O7" t="s">
-        <v>42</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2088,7 +2109,7 @@
         <v>24</v>
       </c>
       <c r="O8" t="s">
-        <v>42</v>
+        <v>202</v>
       </c>
     </row>
     <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2132,7 +2153,7 @@
         <v>24</v>
       </c>
       <c r="O9" t="s">
-        <v>42</v>
+        <v>202</v>
       </c>
     </row>
     <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2176,7 +2197,7 @@
         <v>58</v>
       </c>
       <c r="O10" t="s">
-        <v>59</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2220,7 +2241,7 @@
         <v>24</v>
       </c>
       <c r="O11" t="s">
-        <v>59</v>
+        <v>203</v>
       </c>
     </row>
     <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2264,7 +2285,7 @@
         <v>63</v>
       </c>
       <c r="O12" t="s">
-        <v>59</v>
+        <v>203</v>
       </c>
     </row>
     <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2308,7 +2329,7 @@
         <v>66</v>
       </c>
       <c r="O13" t="s">
-        <v>59</v>
+        <v>203</v>
       </c>
     </row>
     <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2352,7 +2373,7 @@
         <v>24</v>
       </c>
       <c r="O14" t="s">
-        <v>72</v>
+        <v>204</v>
       </c>
     </row>
     <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2396,7 +2417,7 @@
         <v>24</v>
       </c>
       <c r="O15" t="s">
-        <v>72</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2440,7 +2461,7 @@
         <v>24</v>
       </c>
       <c r="O16" t="s">
-        <v>72</v>
+        <v>204</v>
       </c>
     </row>
     <row r="17" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2484,7 +2505,7 @@
         <v>24</v>
       </c>
       <c r="O17" t="s">
-        <v>72</v>
+        <v>204</v>
       </c>
     </row>
     <row r="18" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2528,7 +2549,7 @@
         <v>82</v>
       </c>
       <c r="O18" t="s">
-        <v>72</v>
+        <v>204</v>
       </c>
     </row>
     <row r="19" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2572,7 +2593,7 @@
         <v>24</v>
       </c>
       <c r="O19" t="s">
-        <v>72</v>
+        <v>204</v>
       </c>
     </row>
     <row r="20" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2616,7 +2637,7 @@
         <v>88</v>
       </c>
       <c r="O20" t="s">
-        <v>89</v>
+        <v>205</v>
       </c>
     </row>
     <row r="21" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2660,7 +2681,7 @@
         <v>24</v>
       </c>
       <c r="O21" t="s">
-        <v>89</v>
+        <v>205</v>
       </c>
     </row>
     <row r="22" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2704,7 +2725,7 @@
         <v>92</v>
       </c>
       <c r="O22" t="s">
-        <v>89</v>
+        <v>205</v>
       </c>
     </row>
     <row r="23" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2871,7 +2892,7 @@
         <v>104</v>
       </c>
       <c r="O26" t="s">
-        <v>105</v>
+        <v>206</v>
       </c>
     </row>
     <row r="27" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2915,7 +2936,7 @@
         <v>108</v>
       </c>
       <c r="O27" t="s">
-        <v>105</v>
+        <v>206</v>
       </c>
     </row>
     <row r="28" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -2997,7 +3018,7 @@
         <v>24</v>
       </c>
       <c r="O29" t="s">
-        <v>118</v>
+        <v>207</v>
       </c>
     </row>
     <row r="30" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -3041,7 +3062,7 @@
         <v>24</v>
       </c>
       <c r="O30" t="s">
-        <v>118</v>
+        <v>207</v>
       </c>
     </row>
     <row r="31" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -3261,7 +3282,7 @@
         <v>24</v>
       </c>
       <c r="O35" t="s">
-        <v>137</v>
+        <v>208</v>
       </c>
     </row>
     <row r="36" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -3305,7 +3326,7 @@
         <v>24</v>
       </c>
       <c r="O36" t="s">
-        <v>137</v>
+        <v>208</v>
       </c>
     </row>
     <row r="37" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -3349,7 +3370,7 @@
         <v>24</v>
       </c>
       <c r="O37" t="s">
-        <v>137</v>
+        <v>208</v>
       </c>
     </row>
     <row r="38" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.2">

</xml_diff>